<commit_message>
implement out-of-sample backtesting across multiple horizons
</commit_message>
<xml_diff>
--- a/SA_results_01.xlsx
+++ b/SA_results_01.xlsx
@@ -35,7 +35,7 @@
     <t xml:space="preserve">OK</t>
   </si>
   <si>
-    <t xml:space="preserve">c("AR", "MA", "MA"); c("Nonseasonal", "Nonseasonal", "Seasonal"); c("01", "01", "12"); c("01", "01", "12"); c("+0.31429398576042E+00", "+0.66015567139164E+00", "+0.90098519342969E+00"); c("+0.10708678018301E+00", "+0.84305248208768E-01", "+0.24419866236346E-01"); c("       ", "       ", "       ")</t>
+    <t xml:space="preserve">c("AR", "MA", "MA"); c("Nonseasonal", "Nonseasonal", "Seasonal"); c("01", "01", "12"); c("01", "01", "12"); c("+0.35699023636165E+00", "+0.66748614272404E+00", "+0.97989443623718E+00"); c("+0.10709470702027E+00", "+0.84424755552035E-01", "+0.22352427306943E-01"); c("       ", "       ", "       ")</t>
   </si>
   <si>
     <t xml:space="preserve"/>
@@ -44,31 +44,31 @@
     <t xml:space="preserve">Property tax</t>
   </si>
   <si>
-    <t xml:space="preserve">c("MA", "MA", "MA"); c("Nonseasonal", "Nonseasonal", "Seasonal"); c("01", "01", "12"); c("01", "02", "12"); c("+0.56775056654640E+00", "+0.19229693637269E+00", "+0.88147544290181E+00"); c("+0.51008789273926E-01", "+0.50995722611230E-01", "+0.30580317929367E-01"); c("       ", "       ", "       ")</t>
+    <t xml:space="preserve">c("MA", "MA", "MA"); c("Nonseasonal", "Nonseasonal", "Seasonal"); c("01", "01", "12"); c("01", "02", "12"); c("+0.56968600379091E+00", "+0.18872880275992E+00", "+0.87548449405330E+00"); c("+0.51361175021261E-01", "+0.51363544265612E-01", "+0.31457054960600E-01"); c("       ", "       ", "       ")</t>
   </si>
   <si>
     <t xml:space="preserve">praise tax</t>
   </si>
   <si>
-    <t xml:space="preserve">c("AR", "AR", "AR", "MA", "MA"); c("Nonseasonal", "Nonseasonal", "Nonseasonal", "Nonseasonal", "Seasonal"); c("01", "01", "01", "01", "12"); c("01", "02", "03", "01", "12"); c("+0.74888348640922E-01", "-0.23249104007853E-01", "-0.14359628136814E+00", "+0.58934806026912E+00", "+0.98506927701593E+00"); c("+0.11217200926967E+00", "+0.70474621581935E-01", "+0.61089433085066E-01", "+0.10609067189226E+00", "+0.23124034706061E-01"); c("       ", "       ", "       ", "       ", "       ")</t>
+    <t xml:space="preserve">c("AR", "AR", "AR", "MA", "MA"); c("Nonseasonal", "Nonseasonal", "Nonseasonal", "Nonseasonal", "Seasonal"); c("01", "01", "01", "01", "12"); c("01", "02", "03", "01", "12"); c("+0.79501439805238E-01", "-0.21556516983310E-01", "-0.13775679729727E+00", "+0.59269247305827E+00", "+0.99641858040853E+00"); c("+0.11277895611472E+00", "+0.70629835567064E-01", "+0.61228877515372E-01", "+0.10674504914411E+00", "+0.23886400964421E-01"); c("       ", "       ", "       ", "       ", "       ")</t>
   </si>
   <si>
     <t xml:space="preserve">Real estate purchase tax</t>
   </si>
   <si>
-    <t xml:space="preserve">c("MA", "MA"); c("Nonseasonal", "Seasonal"); c("01", "12"); c("01", "12"); c("+0.38257505232434E+00", "+0.90609562722136E+00"); c("+0.48109958402421E-01", "+0.27474551550903E-01"); c("       ", "       ")</t>
+    <t xml:space="preserve">c("MA", "MA"); c("Nonseasonal", "Seasonal"); c("01", "12"); c("01", "12"); c("+0.38323046727417E+00", "+0.92130368097392E+00"); c("+0.48125158808163E-01", "+0.25681722870265E-01"); c("       ", "       ")</t>
   </si>
   <si>
     <t xml:space="preserve">praise tax returns</t>
   </si>
   <si>
-    <t xml:space="preserve">c("MA", "MA", "MA"); c("Nonseasonal", "Nonseasonal", "Seasonal"); c("01", "01", "12"); c("01", "02", "12"); c("+0.71834912701095E+00", "+0.19547169186854E+00", "+0.87490072788873E+00"); c("+0.50674654200598E-01", "+0.50810872133725E-01", "+0.30948820080718E-01"); c("       ", "       ", "       ")</t>
+    <t xml:space="preserve">c("MA", "MA", "MA"); c("Nonseasonal", "Nonseasonal", "Seasonal"); c("01", "01", "12"); c("01", "02", "12"); c("+0.71736359831315E+00", "+0.19699780988398E+00", "+0.87495777299252E+00"); c("+0.50889884835257E-01", "+0.51031243510684E-01", "+0.31149792543320E-01"); c("       ", "       ", "       ")</t>
   </si>
   <si>
     <t xml:space="preserve">purchase returns</t>
   </si>
   <si>
-    <t xml:space="preserve">c("MA", "MA"); c("Nonseasonal", "Seasonal"); c("01", "12"); c("01", "12"); c("+0.86498302676532E+00", "+0.86273660061665E+00"); c("+0.26545150384317E-01", "+0.32045957398848E-01"); c("       ", "       ")</t>
+    <t xml:space="preserve">c("MA", "MA"); c("Nonseasonal", "Seasonal"); c("01", "12"); c("01", "12"); c("+0.86069166398056E+00", "+0.87549265706783E+00"); c("+0.27123826020871E-01", "+0.30892399983282E-01"); c("       ", "       ")</t>
   </si>
 </sst>
 </file>

</xml_diff>